<commit_message>
Credit author as socragpt across README, CITATION and documents
</commit_message>
<xml_diff>
--- a/openai-hf-2026-instrument.xlsx
+++ b/openai-hf-2026-instrument.xlsx
@@ -43,7 +43,7 @@
     <t xml:space="preserve">Worked example: The OpenAI–Hugging Face Incident (April–July 2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">Version 1.0  ·  31 August 2026  ·  Author: Tyler Pearson  ·  Licence: CC BY-SA 4.0</t>
+    <t xml:space="preserve">Version 1.0  ·  31 August 2026  ·  Author: socragpt  ·  Licence: CC BY-SA 4.0</t>
   </si>
   <si>
     <t xml:space="preserve">An independent, open RCSA instrument: a standard self-assessment method for the frontier-model evaluation process, shipped populated with a worked example drawn from a real, publicly documented incident. Not affiliated with, authorised by, or endorsed by OpenAI or Hugging Face. Ratings are the author's own and are indicative.</t>
@@ -196,7 +196,7 @@
     <t xml:space="preserve">Approves residual risk &amp; action plan</t>
   </si>
   <si>
-    <t xml:space="preserve">Legend — cells shaded pale yellow are for completion by the assessor. In the register and library tabs, white data cells are editable; grey/navy headers and the calculated columns (scores, bands, appetite status, priority) are driven by formulas. © 2026 Tyler Pearson. Licensed under CC BY-SA 4.0.</t>
+    <t xml:space="preserve">Legend — cells shaded pale yellow are for completion by the assessor. In the register and library tabs, white data cells are editable; grey/navy headers and the calculated columns (scores, bands, appetite status, priority) are driven by formulas. © 2026 socragpt. Licensed under CC BY-SA 4.0.</t>
   </si>
   <si>
     <t xml:space="preserve">Methodology &amp; Risk Appetite</t>

</xml_diff>

<commit_message>
Relicense to CC BY 4.0 (LICENSE, README, CITATION, documents)
</commit_message>
<xml_diff>
--- a/openai-hf-2026-instrument.xlsx
+++ b/openai-hf-2026-instrument.xlsx
@@ -43,7 +43,7 @@
     <t xml:space="preserve">Worked example: The OpenAI–Hugging Face Incident (April–July 2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">Version 1.0  ·  31 August 2026  ·  Author: socragpt  ·  Licence: CC BY-SA 4.0</t>
+    <t xml:space="preserve">Version 1.0  ·  31 August 2026  ·  Author: socragpt  ·  Licence: CC BY 4.0</t>
   </si>
   <si>
     <t xml:space="preserve">An independent, open RCSA instrument: a standard self-assessment method for the frontier-model evaluation process, shipped populated with a worked example drawn from a real, publicly documented incident. Not affiliated with, authorised by, or endorsed by OpenAI or Hugging Face. Ratings are the author's own and are indicative.</t>
@@ -196,7 +196,7 @@
     <t xml:space="preserve">Approves residual risk &amp; action plan</t>
   </si>
   <si>
-    <t xml:space="preserve">Legend — cells shaded pale yellow are for completion by the assessor. In the register and library tabs, white data cells are editable; grey/navy headers and the calculated columns (scores, bands, appetite status, priority) are driven by formulas. © 2026 socragpt. Licensed under CC BY-SA 4.0.</t>
+    <t xml:space="preserve">Legend — cells shaded pale yellow are for completion by the assessor. In the register and library tabs, white data cells are editable; grey/navy headers and the calculated columns (scores, bands, appetite status, priority) are driven by formulas. © 2026 socragpt. Licensed under CC BY 4.0.</t>
   </si>
   <si>
     <t xml:space="preserve">Methodology &amp; Risk Appetite</t>

</xml_diff>